<commit_message>
backup: before judge-sheet print performance optimization
</commit_message>
<xml_diff>
--- a/仕様書/帳票一覧.xlsx
+++ b/仕様書/帳票一覧.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\JDSF\DScore\DSPrt\仕様書\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CC0AA09-3F06-4FC4-A5ED-D8E12E3BCEE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50246513-2702-4F8A-8504-DA438A45A198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4704" yWindow="2292" windowWidth="28980" windowHeight="14496" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1536" yWindow="6960" windowWidth="28980" windowHeight="14496" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2780,12 +2780,24 @@
       <c r="J5" s="40">
         <v>1</v>
       </c>
-      <c r="K5" s="44"/>
-      <c r="L5" s="10"/>
-      <c r="M5" s="11"/>
-      <c r="N5" s="31"/>
-      <c r="O5" s="10"/>
-      <c r="P5" s="11"/>
+      <c r="K5" s="44">
+        <v>1</v>
+      </c>
+      <c r="L5" s="10">
+        <v>1</v>
+      </c>
+      <c r="M5" s="11">
+        <v>1</v>
+      </c>
+      <c r="N5" s="31">
+        <v>1</v>
+      </c>
+      <c r="O5" s="10">
+        <v>1</v>
+      </c>
+      <c r="P5" s="11">
+        <v>1</v>
+      </c>
     </row>
     <row r="6" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B6" s="12"/>
@@ -2983,13 +2995,19 @@
       <c r="G11" s="58" t="s">
         <v>81</v>
       </c>
-      <c r="H11" s="59"/>
+      <c r="H11" s="59">
+        <v>1</v>
+      </c>
       <c r="I11" s="60"/>
       <c r="J11" s="61"/>
-      <c r="K11" s="62"/>
+      <c r="K11" s="62">
+        <v>1</v>
+      </c>
       <c r="L11" s="60"/>
       <c r="M11" s="63"/>
-      <c r="N11" s="59"/>
+      <c r="N11" s="59">
+        <v>1</v>
+      </c>
       <c r="O11" s="60"/>
       <c r="P11" s="63"/>
     </row>

</xml_diff>